<commit_message>
implementação segunda guia FICHA RECADASTRO V.2026-2.xlsx"
</commit_message>
<xml_diff>
--- a/backend/assets/FICHA RECADASTRO V.2026-2.xlsx
+++ b/backend/assets/FICHA RECADASTRO V.2026-2.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,22 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\OrderSync\backend\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76790FE3-A557-4483-A191-38EA82768E0D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB918709-CA4D-459C-876C-A7F84A8ED4D5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33210" yWindow="1485" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro Parte 1" sheetId="5" r:id="rId1"/>
+    <sheet name="Cadastro Parte 2" sheetId="6" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Cadastro Parte 1'!$A$1:$K$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Cadastro Parte 2'!$A$1:$K$8</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="83">
   <si>
     <t>COMERCIAL</t>
   </si>
@@ -273,12 +275,78 @@
   <si>
     <t>v.2026/02</t>
   </si>
+  <si>
+    <t>Referências Comerciais</t>
+  </si>
+  <si>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade </t>
+  </si>
+  <si>
+    <t>Bens Imóveis</t>
+  </si>
+  <si>
+    <t>Imóvel</t>
+  </si>
+  <si>
+    <t>Localização</t>
+  </si>
+  <si>
+    <t>Área</t>
+  </si>
+  <si>
+    <t>Valor  (R$)</t>
+  </si>
+  <si>
+    <t>Hipotecado</t>
+  </si>
+  <si>
+    <t>Plantel de Animais</t>
+  </si>
+  <si>
+    <t>Espécie</t>
+  </si>
+  <si>
+    <t>Nº de Animais</t>
+  </si>
+  <si>
+    <t>Consumo Médio Diário (Kg)</t>
+  </si>
+  <si>
+    <t>Consumo Médio Mensal (Kg)</t>
+  </si>
+  <si>
+    <t>Bens Móveis (Veículos/Máquinas/Equipamentos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marca </t>
+  </si>
+  <si>
+    <t>Modelo</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Alienado</t>
+  </si>
+  <si>
+    <t>Nome do Cliente :</t>
+  </si>
+  <si>
+    <t>Código do Cliente :</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -352,16 +420,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="59">
+  <borders count="61">
     <border>
       <left/>
       <right/>
@@ -1077,11 +1158,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="226">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1196,6 +1301,366 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1226,15 +1691,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1244,355 +1700,139 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1829,6 +2069,85 @@
         <a:xfrm>
           <a:off x="5657850" y="8858250"/>
           <a:ext cx="1228725" cy="1228725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A660AC1D-25FC-4D19-9682-60C63B83CEED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="219075" y="57150"/>
+          <a:ext cx="1295400" cy="619125"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2183,7 +2502,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2210,27 +2529,27 @@
     </row>
     <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="25"/>
-      <c r="D2" s="66" t="s">
+      <c r="D2" s="152" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="67"/>
+      <c r="E2" s="152"/>
+      <c r="F2" s="152"/>
+      <c r="G2" s="152"/>
+      <c r="H2" s="152"/>
+      <c r="I2" s="152"/>
+      <c r="J2" s="152"/>
+      <c r="K2" s="153"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="67"/>
+      <c r="D3" s="152"/>
+      <c r="E3" s="152"/>
+      <c r="F3" s="152"/>
+      <c r="G3" s="152"/>
+      <c r="H3" s="152"/>
+      <c r="I3" s="152"/>
+      <c r="J3" s="152"/>
+      <c r="K3" s="153"/>
     </row>
     <row r="4" spans="1:11" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17"/>
@@ -2252,50 +2571,50 @@
       <c r="K5" s="30"/>
     </row>
     <row r="6" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="174" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="54" t="s">
+      <c r="B6" s="175"/>
+      <c r="C6" s="175"/>
+      <c r="D6" s="175"/>
+      <c r="E6" s="175"/>
+      <c r="F6" s="175"/>
+      <c r="G6" s="175"/>
+      <c r="H6" s="175"/>
+      <c r="I6" s="174" t="s">
         <v>1</v>
       </c>
-      <c r="J6" s="55"/>
-      <c r="K6" s="56"/>
+      <c r="J6" s="175"/>
+      <c r="K6" s="176"/>
     </row>
     <row r="7" spans="1:11" s="6" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="80" t="s">
+      <c r="A7" s="164" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="81"/>
-      <c r="C7" s="81"/>
-      <c r="D7" s="81"/>
-      <c r="E7" s="81"/>
-      <c r="F7" s="81"/>
-      <c r="G7" s="81"/>
-      <c r="H7" s="82"/>
-      <c r="I7" s="71" t="s">
+      <c r="B7" s="165"/>
+      <c r="C7" s="165"/>
+      <c r="D7" s="165"/>
+      <c r="E7" s="165"/>
+      <c r="F7" s="165"/>
+      <c r="G7" s="165"/>
+      <c r="H7" s="166"/>
+      <c r="I7" s="157" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="72"/>
-      <c r="K7" s="73"/>
+      <c r="J7" s="158"/>
+      <c r="K7" s="159"/>
     </row>
     <row r="8" spans="1:11" s="6" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="160" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="76"/>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
-      <c r="F8" s="76"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="77"/>
+      <c r="B8" s="161"/>
+      <c r="C8" s="162"/>
+      <c r="D8" s="162"/>
+      <c r="E8" s="162"/>
+      <c r="F8" s="162"/>
+      <c r="G8" s="162"/>
+      <c r="H8" s="163"/>
       <c r="I8" s="7"/>
       <c r="J8" s="8"/>
       <c r="K8" s="9"/>
@@ -2306,11 +2625,11 @@
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
-      <c r="D9" s="78"/>
-      <c r="E9" s="78"/>
-      <c r="F9" s="78"/>
-      <c r="G9" s="78"/>
-      <c r="H9" s="79"/>
+      <c r="D9" s="95"/>
+      <c r="E9" s="95"/>
+      <c r="F9" s="95"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="96"/>
       <c r="I9" s="7" t="s">
         <v>6</v>
       </c>
@@ -2318,100 +2637,100 @@
       <c r="K9" s="9"/>
     </row>
     <row r="10" spans="1:11" s="6" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="104" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="84"/>
-      <c r="C10" s="84"/>
-      <c r="D10" s="84"/>
-      <c r="E10" s="84"/>
-      <c r="F10" s="84"/>
-      <c r="G10" s="84"/>
-      <c r="H10" s="85"/>
+      <c r="B10" s="105"/>
+      <c r="C10" s="105"/>
+      <c r="D10" s="105"/>
+      <c r="E10" s="105"/>
+      <c r="F10" s="105"/>
+      <c r="G10" s="105"/>
+      <c r="H10" s="167"/>
       <c r="I10" s="12"/>
       <c r="J10" s="13"/>
       <c r="K10" s="14"/>
     </row>
     <row r="11" spans="1:11" s="6" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="59" t="s">
+      <c r="A11" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="68" t="s">
+      <c r="B11" s="82"/>
+      <c r="C11" s="82"/>
+      <c r="D11" s="82"/>
+      <c r="E11" s="154" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="69"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="69"/>
-      <c r="J11" s="69"/>
-      <c r="K11" s="70"/>
+      <c r="F11" s="155"/>
+      <c r="G11" s="155"/>
+      <c r="H11" s="155"/>
+      <c r="I11" s="155"/>
+      <c r="J11" s="155"/>
+      <c r="K11" s="156"/>
     </row>
     <row r="12" spans="1:11" s="6" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="59" t="s">
+      <c r="A12" s="81" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="61" t="s">
+      <c r="B12" s="82"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="178" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="62"/>
+      <c r="F12" s="178"/>
+      <c r="G12" s="178"/>
+      <c r="H12" s="178"/>
+      <c r="I12" s="178"/>
+      <c r="J12" s="178"/>
+      <c r="K12" s="179"/>
     </row>
     <row r="13" spans="1:11" s="6" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="180" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="64"/>
-      <c r="C13" s="64"/>
-      <c r="D13" s="64"/>
-      <c r="E13" s="64" t="s">
+      <c r="B13" s="150"/>
+      <c r="C13" s="150"/>
+      <c r="D13" s="150"/>
+      <c r="E13" s="150" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="64"/>
-      <c r="G13" s="64"/>
-      <c r="H13" s="64"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="64"/>
-      <c r="K13" s="65"/>
+      <c r="F13" s="150"/>
+      <c r="G13" s="150"/>
+      <c r="H13" s="150"/>
+      <c r="I13" s="150"/>
+      <c r="J13" s="150"/>
+      <c r="K13" s="151"/>
     </row>
     <row r="14" spans="1:11" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="51" t="s">
+      <c r="A14" s="171" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="52"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="52"/>
-      <c r="I14" s="52"/>
-      <c r="J14" s="52"/>
-      <c r="K14" s="53"/>
+      <c r="B14" s="172"/>
+      <c r="C14" s="172"/>
+      <c r="D14" s="172"/>
+      <c r="E14" s="172"/>
+      <c r="F14" s="172"/>
+      <c r="G14" s="172"/>
+      <c r="H14" s="172"/>
+      <c r="I14" s="172"/>
+      <c r="J14" s="172"/>
+      <c r="K14" s="173"/>
     </row>
     <row r="15" spans="1:11" s="6" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="168" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="50"/>
+      <c r="B15" s="169"/>
+      <c r="C15" s="169"/>
+      <c r="D15" s="169"/>
+      <c r="E15" s="169"/>
+      <c r="F15" s="169"/>
+      <c r="G15" s="169"/>
+      <c r="H15" s="169"/>
+      <c r="I15" s="169"/>
+      <c r="J15" s="169"/>
+      <c r="K15" s="170"/>
     </row>
     <row r="16" spans="1:11" s="6" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="27"/>
@@ -2427,19 +2746,19 @@
       <c r="K16" s="21"/>
     </row>
     <row r="17" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="126" t="s">
+      <c r="A17" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="127"/>
-      <c r="C17" s="127"/>
-      <c r="D17" s="127"/>
-      <c r="E17" s="127"/>
-      <c r="F17" s="127"/>
-      <c r="G17" s="127"/>
-      <c r="H17" s="127"/>
-      <c r="I17" s="127"/>
-      <c r="J17" s="127"/>
-      <c r="K17" s="128"/>
+      <c r="B17" s="98"/>
+      <c r="C17" s="98"/>
+      <c r="D17" s="98"/>
+      <c r="E17" s="98"/>
+      <c r="F17" s="98"/>
+      <c r="G17" s="98"/>
+      <c r="H17" s="98"/>
+      <c r="I17" s="98"/>
+      <c r="J17" s="98"/>
+      <c r="K17" s="99"/>
     </row>
     <row r="18" spans="1:16" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31"/>
@@ -2455,55 +2774,55 @@
       <c r="K18" s="28"/>
     </row>
     <row r="19" spans="1:16" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="86" t="s">
+      <c r="A19" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="87"/>
-      <c r="C19" s="87"/>
-      <c r="D19" s="87"/>
-      <c r="E19" s="87"/>
-      <c r="F19" s="87"/>
-      <c r="G19" s="87"/>
-      <c r="H19" s="87"/>
-      <c r="I19" s="87"/>
-      <c r="J19" s="87"/>
-      <c r="K19" s="88"/>
+      <c r="B19" s="127"/>
+      <c r="C19" s="127"/>
+      <c r="D19" s="127"/>
+      <c r="E19" s="127"/>
+      <c r="F19" s="127"/>
+      <c r="G19" s="127"/>
+      <c r="H19" s="127"/>
+      <c r="I19" s="127"/>
+      <c r="J19" s="127"/>
+      <c r="K19" s="128"/>
     </row>
     <row r="20" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="93" t="s">
+      <c r="A20" s="147" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="94"/>
-      <c r="C20" s="94"/>
-      <c r="D20" s="94"/>
-      <c r="E20" s="94"/>
-      <c r="F20" s="94"/>
-      <c r="G20" s="94"/>
-      <c r="H20" s="95"/>
-      <c r="I20" s="96" t="s">
+      <c r="B20" s="148"/>
+      <c r="C20" s="148"/>
+      <c r="D20" s="148"/>
+      <c r="E20" s="148"/>
+      <c r="F20" s="148"/>
+      <c r="G20" s="148"/>
+      <c r="H20" s="149"/>
+      <c r="I20" s="137" t="s">
         <v>25</v>
       </c>
-      <c r="J20" s="97"/>
-      <c r="K20" s="98"/>
+      <c r="J20" s="138"/>
+      <c r="K20" s="139"/>
     </row>
     <row r="21" spans="1:16" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="99" t="s">
+      <c r="A21" s="140" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="90"/>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="89" t="s">
+      <c r="B21" s="141"/>
+      <c r="C21" s="141"/>
+      <c r="D21" s="141"/>
+      <c r="E21" s="141"/>
+      <c r="F21" s="142" t="s">
         <v>30</v>
       </c>
-      <c r="G21" s="90"/>
-      <c r="H21" s="91"/>
-      <c r="I21" s="89" t="s">
+      <c r="G21" s="141"/>
+      <c r="H21" s="143"/>
+      <c r="I21" s="142" t="s">
         <v>26</v>
       </c>
-      <c r="J21" s="90"/>
-      <c r="K21" s="92"/>
+      <c r="J21" s="141"/>
+      <c r="K21" s="144"/>
     </row>
     <row r="22" spans="1:16" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="31"/>
@@ -2519,55 +2838,55 @@
       <c r="K22" s="29"/>
     </row>
     <row r="23" spans="1:16" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="86" t="s">
+      <c r="A23" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="87"/>
-      <c r="C23" s="87"/>
-      <c r="D23" s="87"/>
-      <c r="E23" s="87"/>
-      <c r="F23" s="87"/>
-      <c r="G23" s="87"/>
-      <c r="H23" s="87"/>
-      <c r="I23" s="87"/>
-      <c r="J23" s="87"/>
-      <c r="K23" s="88"/>
+      <c r="B23" s="127"/>
+      <c r="C23" s="127"/>
+      <c r="D23" s="127"/>
+      <c r="E23" s="127"/>
+      <c r="F23" s="127"/>
+      <c r="G23" s="127"/>
+      <c r="H23" s="127"/>
+      <c r="I23" s="127"/>
+      <c r="J23" s="127"/>
+      <c r="K23" s="128"/>
     </row>
     <row r="24" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="102" t="s">
+      <c r="A24" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="103"/>
-      <c r="C24" s="103"/>
-      <c r="D24" s="103"/>
-      <c r="E24" s="103"/>
-      <c r="F24" s="103"/>
-      <c r="G24" s="103"/>
-      <c r="H24" s="104"/>
-      <c r="I24" s="96" t="s">
+      <c r="B24" s="135"/>
+      <c r="C24" s="135"/>
+      <c r="D24" s="135"/>
+      <c r="E24" s="135"/>
+      <c r="F24" s="135"/>
+      <c r="G24" s="135"/>
+      <c r="H24" s="136"/>
+      <c r="I24" s="137" t="s">
         <v>25</v>
       </c>
-      <c r="J24" s="97"/>
-      <c r="K24" s="98"/>
+      <c r="J24" s="138"/>
+      <c r="K24" s="139"/>
     </row>
     <row r="25" spans="1:16" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="99" t="s">
+      <c r="A25" s="140" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="90"/>
-      <c r="C25" s="90"/>
-      <c r="D25" s="90"/>
-      <c r="E25" s="90"/>
-      <c r="F25" s="89" t="s">
+      <c r="B25" s="141"/>
+      <c r="C25" s="141"/>
+      <c r="D25" s="141"/>
+      <c r="E25" s="141"/>
+      <c r="F25" s="142" t="s">
         <v>30</v>
       </c>
-      <c r="G25" s="90"/>
-      <c r="H25" s="91"/>
-      <c r="I25" s="89" t="s">
+      <c r="G25" s="141"/>
+      <c r="H25" s="143"/>
+      <c r="I25" s="142" t="s">
         <v>28</v>
       </c>
-      <c r="J25" s="90"/>
-      <c r="K25" s="92"/>
+      <c r="J25" s="141"/>
+      <c r="K25" s="144"/>
     </row>
     <row r="26" spans="1:16" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="31"/>
@@ -2583,19 +2902,19 @@
       <c r="K26" s="29"/>
     </row>
     <row r="27" spans="1:16" s="1" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="86" t="s">
+      <c r="A27" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="172"/>
-      <c r="C27" s="173"/>
-      <c r="D27" s="174"/>
-      <c r="E27" s="174"/>
-      <c r="F27" s="174"/>
-      <c r="G27" s="174"/>
-      <c r="H27" s="174"/>
-      <c r="I27" s="174"/>
-      <c r="J27" s="174"/>
-      <c r="K27" s="175"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
+      <c r="I27" s="54"/>
+      <c r="J27" s="54"/>
+      <c r="K27" s="55"/>
     </row>
     <row r="28" spans="1:16" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="45"/>
@@ -2611,180 +2930,180 @@
       <c r="K28" s="47"/>
     </row>
     <row r="29" spans="1:16" s="1" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="86" t="s">
+      <c r="A29" s="51" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="87"/>
-      <c r="C29" s="87"/>
-      <c r="D29" s="87"/>
-      <c r="E29" s="87"/>
-      <c r="F29" s="87"/>
-      <c r="G29" s="87"/>
-      <c r="H29" s="87"/>
-      <c r="I29" s="87"/>
-      <c r="J29" s="87"/>
-      <c r="K29" s="88"/>
+      <c r="B29" s="127"/>
+      <c r="C29" s="127"/>
+      <c r="D29" s="127"/>
+      <c r="E29" s="127"/>
+      <c r="F29" s="127"/>
+      <c r="G29" s="127"/>
+      <c r="H29" s="127"/>
+      <c r="I29" s="127"/>
+      <c r="J29" s="127"/>
+      <c r="K29" s="128"/>
     </row>
     <row r="30" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="105" t="s">
+      <c r="A30" s="145" t="s">
         <v>10</v>
       </c>
-      <c r="B30" s="106"/>
-      <c r="C30" s="101" t="s">
+      <c r="B30" s="146"/>
+      <c r="C30" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="101"/>
-      <c r="E30" s="101" t="s">
+      <c r="D30" s="72"/>
+      <c r="E30" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="101"/>
+      <c r="F30" s="72"/>
       <c r="G30" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="H30" s="101" t="s">
+      <c r="H30" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="I30" s="101"/>
-      <c r="J30" s="101" t="s">
+      <c r="I30" s="72"/>
+      <c r="J30" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="K30" s="110"/>
+      <c r="K30" s="130"/>
     </row>
     <row r="31" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="107" t="s">
+      <c r="A31" s="125" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="108"/>
-      <c r="C31" s="112"/>
-      <c r="D31" s="113"/>
-      <c r="E31" s="112"/>
-      <c r="F31" s="113"/>
+      <c r="B31" s="126"/>
+      <c r="C31" s="132"/>
+      <c r="D31" s="133"/>
+      <c r="E31" s="132"/>
+      <c r="F31" s="133"/>
       <c r="G31" s="35"/>
-      <c r="H31" s="109"/>
-      <c r="I31" s="109"/>
-      <c r="J31" s="109"/>
-      <c r="K31" s="111"/>
+      <c r="H31" s="129"/>
+      <c r="I31" s="129"/>
+      <c r="J31" s="129"/>
+      <c r="K31" s="131"/>
       <c r="P31" s="2"/>
     </row>
     <row r="32" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="107" t="s">
+      <c r="A32" s="125" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="108"/>
-      <c r="C32" s="100"/>
-      <c r="D32" s="100"/>
-      <c r="E32" s="100"/>
-      <c r="F32" s="100"/>
+      <c r="B32" s="126"/>
+      <c r="C32" s="120"/>
+      <c r="D32" s="120"/>
+      <c r="E32" s="120"/>
+      <c r="F32" s="120"/>
       <c r="G32" s="33"/>
-      <c r="H32" s="100"/>
-      <c r="I32" s="100"/>
-      <c r="J32" s="100"/>
+      <c r="H32" s="120"/>
+      <c r="I32" s="120"/>
+      <c r="J32" s="120"/>
       <c r="K32" s="121"/>
     </row>
     <row r="33" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="124" t="s">
+      <c r="A33" s="123" t="s">
         <v>19</v>
       </c>
-      <c r="B33" s="125"/>
-      <c r="C33" s="122"/>
-      <c r="D33" s="122"/>
-      <c r="E33" s="122"/>
-      <c r="F33" s="122"/>
+      <c r="B33" s="124"/>
+      <c r="C33" s="112"/>
+      <c r="D33" s="112"/>
+      <c r="E33" s="112"/>
+      <c r="F33" s="112"/>
       <c r="G33" s="34"/>
-      <c r="H33" s="122"/>
-      <c r="I33" s="122"/>
-      <c r="J33" s="122"/>
-      <c r="K33" s="123"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+      <c r="J33" s="112"/>
+      <c r="K33" s="122"/>
     </row>
     <row r="34" spans="1:11" s="1" customFormat="1" ht="3" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="169"/>
-      <c r="B34" s="170"/>
-      <c r="C34" s="170"/>
-      <c r="D34" s="170"/>
-      <c r="E34" s="170"/>
-      <c r="F34" s="170"/>
-      <c r="G34" s="170"/>
-      <c r="H34" s="170"/>
-      <c r="I34" s="170"/>
-      <c r="J34" s="170"/>
-      <c r="K34" s="171"/>
+      <c r="A34" s="48"/>
+      <c r="B34" s="49"/>
+      <c r="C34" s="49"/>
+      <c r="D34" s="49"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="49"/>
+      <c r="H34" s="49"/>
+      <c r="I34" s="49"/>
+      <c r="J34" s="49"/>
+      <c r="K34" s="50"/>
     </row>
     <row r="35" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="129" t="s">
+      <c r="A35" s="100" t="s">
         <v>46</v>
       </c>
-      <c r="B35" s="130"/>
-      <c r="C35" s="131"/>
-      <c r="D35" s="131"/>
-      <c r="E35" s="131"/>
-      <c r="F35" s="131"/>
-      <c r="G35" s="131"/>
-      <c r="H35" s="131"/>
-      <c r="I35" s="131"/>
-      <c r="J35" s="131"/>
-      <c r="K35" s="132"/>
+      <c r="B35" s="59"/>
+      <c r="C35" s="101"/>
+      <c r="D35" s="101"/>
+      <c r="E35" s="101"/>
+      <c r="F35" s="101"/>
+      <c r="G35" s="101"/>
+      <c r="H35" s="101"/>
+      <c r="I35" s="101"/>
+      <c r="J35" s="101"/>
+      <c r="K35" s="102"/>
     </row>
     <row r="36" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="133" t="s">
+      <c r="A36" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="134"/>
-      <c r="C36" s="143" t="s">
+      <c r="B36" s="103"/>
+      <c r="C36" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="D36" s="144"/>
-      <c r="E36" s="144"/>
-      <c r="F36" s="144"/>
-      <c r="G36" s="144"/>
-      <c r="H36" s="144"/>
-      <c r="I36" s="144"/>
-      <c r="J36" s="144"/>
-      <c r="K36" s="145"/>
+      <c r="D36" s="87"/>
+      <c r="E36" s="87"/>
+      <c r="F36" s="87"/>
+      <c r="G36" s="87"/>
+      <c r="H36" s="87"/>
+      <c r="I36" s="87"/>
+      <c r="J36" s="87"/>
+      <c r="K36" s="88"/>
     </row>
     <row r="37" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="83" t="s">
+      <c r="A37" s="104" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="84"/>
-      <c r="C37" s="146"/>
-      <c r="D37" s="147"/>
-      <c r="E37" s="147"/>
-      <c r="F37" s="147"/>
-      <c r="G37" s="147"/>
-      <c r="H37" s="147"/>
-      <c r="I37" s="147"/>
-      <c r="J37" s="147"/>
-      <c r="K37" s="148"/>
+      <c r="B37" s="105"/>
+      <c r="C37" s="89"/>
+      <c r="D37" s="90"/>
+      <c r="E37" s="90"/>
+      <c r="F37" s="90"/>
+      <c r="G37" s="90"/>
+      <c r="H37" s="90"/>
+      <c r="I37" s="90"/>
+      <c r="J37" s="90"/>
+      <c r="K37" s="91"/>
     </row>
     <row r="38" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="83" t="s">
+      <c r="A38" s="104" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="84"/>
-      <c r="C38" s="146"/>
-      <c r="D38" s="147"/>
-      <c r="E38" s="147"/>
-      <c r="F38" s="147"/>
-      <c r="G38" s="147"/>
-      <c r="H38" s="147"/>
-      <c r="I38" s="147"/>
-      <c r="J38" s="147"/>
-      <c r="K38" s="148"/>
+      <c r="B38" s="105"/>
+      <c r="C38" s="89"/>
+      <c r="D38" s="90"/>
+      <c r="E38" s="90"/>
+      <c r="F38" s="90"/>
+      <c r="G38" s="90"/>
+      <c r="H38" s="90"/>
+      <c r="I38" s="90"/>
+      <c r="J38" s="90"/>
+      <c r="K38" s="91"/>
     </row>
     <row r="39" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="139" t="s">
+      <c r="A39" s="110" t="s">
         <v>41</v>
       </c>
-      <c r="B39" s="140"/>
-      <c r="C39" s="149"/>
-      <c r="D39" s="150"/>
-      <c r="E39" s="150"/>
-      <c r="F39" s="150"/>
-      <c r="G39" s="150"/>
-      <c r="H39" s="150"/>
-      <c r="I39" s="150"/>
-      <c r="J39" s="150"/>
-      <c r="K39" s="151"/>
+      <c r="B39" s="111"/>
+      <c r="C39" s="92"/>
+      <c r="D39" s="93"/>
+      <c r="E39" s="93"/>
+      <c r="F39" s="93"/>
+      <c r="G39" s="93"/>
+      <c r="H39" s="93"/>
+      <c r="I39" s="93"/>
+      <c r="J39" s="93"/>
+      <c r="K39" s="94"/>
     </row>
     <row r="40" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="37"/>
@@ -2800,83 +3119,83 @@
       <c r="K40" s="44"/>
     </row>
     <row r="41" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="152" t="s">
+      <c r="A41" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="153"/>
-      <c r="C41" s="153"/>
-      <c r="D41" s="153"/>
-      <c r="E41" s="153"/>
-      <c r="F41" s="153"/>
-      <c r="G41" s="153"/>
-      <c r="H41" s="153"/>
-      <c r="I41" s="153"/>
-      <c r="J41" s="153"/>
-      <c r="K41" s="154"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="63"/>
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="66"/>
     </row>
     <row r="42" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="133" t="s">
+      <c r="A42" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="B42" s="179"/>
-      <c r="C42" s="78" t="s">
+      <c r="B42" s="61"/>
+      <c r="C42" s="95" t="s">
         <v>59</v>
       </c>
-      <c r="D42" s="78"/>
-      <c r="E42" s="78"/>
-      <c r="F42" s="78"/>
-      <c r="G42" s="78"/>
-      <c r="H42" s="78"/>
-      <c r="I42" s="78"/>
-      <c r="J42" s="78"/>
-      <c r="K42" s="79"/>
+      <c r="D42" s="95"/>
+      <c r="E42" s="95"/>
+      <c r="F42" s="95"/>
+      <c r="G42" s="95"/>
+      <c r="H42" s="95"/>
+      <c r="I42" s="95"/>
+      <c r="J42" s="95"/>
+      <c r="K42" s="96"/>
     </row>
     <row r="43" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="59" t="s">
+      <c r="A43" s="81" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="60"/>
-      <c r="C43" s="57" t="s">
+      <c r="B43" s="82"/>
+      <c r="C43" s="177" t="s">
         <v>60</v>
       </c>
-      <c r="D43" s="57"/>
-      <c r="E43" s="57"/>
-      <c r="F43" s="57"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
+      <c r="D43" s="177"/>
+      <c r="E43" s="177"/>
+      <c r="F43" s="177"/>
+      <c r="G43" s="177"/>
+      <c r="H43" s="177"/>
+      <c r="I43" s="177"/>
+      <c r="J43" s="177"/>
+      <c r="K43" s="177"/>
     </row>
     <row r="44" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="59" t="s">
+      <c r="A44" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="60"/>
-      <c r="C44" s="58"/>
-      <c r="D44" s="58"/>
-      <c r="E44" s="58"/>
-      <c r="F44" s="58"/>
-      <c r="G44" s="58"/>
-      <c r="H44" s="58"/>
-      <c r="I44" s="58"/>
-      <c r="J44" s="58"/>
-      <c r="K44" s="58"/>
+      <c r="B44" s="82"/>
+      <c r="C44" s="85"/>
+      <c r="D44" s="85"/>
+      <c r="E44" s="85"/>
+      <c r="F44" s="85"/>
+      <c r="G44" s="85"/>
+      <c r="H44" s="85"/>
+      <c r="I44" s="85"/>
+      <c r="J44" s="85"/>
+      <c r="K44" s="85"/>
     </row>
     <row r="45" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="141" t="s">
+      <c r="A45" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="B45" s="142"/>
-      <c r="C45" s="58"/>
-      <c r="D45" s="58"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="58"/>
-      <c r="G45" s="58"/>
-      <c r="H45" s="58"/>
-      <c r="I45" s="58"/>
-      <c r="J45" s="58"/>
-      <c r="K45" s="58"/>
+      <c r="B45" s="84"/>
+      <c r="C45" s="85"/>
+      <c r="D45" s="85"/>
+      <c r="E45" s="85"/>
+      <c r="F45" s="85"/>
+      <c r="G45" s="85"/>
+      <c r="H45" s="85"/>
+      <c r="I45" s="85"/>
+      <c r="J45" s="85"/>
+      <c r="K45" s="85"/>
     </row>
     <row r="46" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="37"/>
@@ -2892,102 +3211,102 @@
       <c r="K46" s="40"/>
     </row>
     <row r="47" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="152" t="s">
+      <c r="A47" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="153"/>
-      <c r="C47" s="153"/>
-      <c r="D47" s="180"/>
-      <c r="E47" s="155" t="s">
+      <c r="B47" s="63"/>
+      <c r="C47" s="63"/>
+      <c r="D47" s="64"/>
+      <c r="E47" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="F47" s="153"/>
-      <c r="G47" s="180"/>
-      <c r="H47" s="155" t="s">
+      <c r="F47" s="63"/>
+      <c r="G47" s="64"/>
+      <c r="H47" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="I47" s="153"/>
-      <c r="J47" s="153"/>
-      <c r="K47" s="154"/>
+      <c r="I47" s="63"/>
+      <c r="J47" s="63"/>
+      <c r="K47" s="66"/>
     </row>
     <row r="48" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="156" t="s">
+      <c r="A48" s="67" t="s">
         <v>50</v>
       </c>
-      <c r="B48" s="157"/>
-      <c r="C48" s="160" t="s">
+      <c r="B48" s="68"/>
+      <c r="C48" s="71" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="160"/>
-      <c r="E48" s="101"/>
-      <c r="F48" s="101"/>
-      <c r="G48" s="101"/>
-      <c r="H48" s="161"/>
-      <c r="I48" s="162"/>
-      <c r="J48" s="162"/>
-      <c r="K48" s="163"/>
+      <c r="D48" s="71"/>
+      <c r="E48" s="72"/>
+      <c r="F48" s="72"/>
+      <c r="G48" s="72"/>
+      <c r="H48" s="73"/>
+      <c r="I48" s="74"/>
+      <c r="J48" s="74"/>
+      <c r="K48" s="75"/>
     </row>
     <row r="49" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="158"/>
-      <c r="B49" s="159"/>
-      <c r="C49" s="164" t="s">
+      <c r="A49" s="69"/>
+      <c r="B49" s="70"/>
+      <c r="C49" s="76" t="s">
         <v>52</v>
       </c>
-      <c r="D49" s="164"/>
-      <c r="E49" s="165"/>
-      <c r="F49" s="166"/>
-      <c r="G49" s="167"/>
-      <c r="H49" s="165"/>
-      <c r="I49" s="166"/>
-      <c r="J49" s="166"/>
-      <c r="K49" s="168"/>
+      <c r="D49" s="76"/>
+      <c r="E49" s="77"/>
+      <c r="F49" s="78"/>
+      <c r="G49" s="79"/>
+      <c r="H49" s="77"/>
+      <c r="I49" s="78"/>
+      <c r="J49" s="78"/>
+      <c r="K49" s="80"/>
     </row>
     <row r="50" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="176" t="s">
+      <c r="A50" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="177"/>
-      <c r="C50" s="178" t="s">
+      <c r="B50" s="57"/>
+      <c r="C50" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="D50" s="178"/>
-      <c r="E50" s="130"/>
-      <c r="F50" s="130"/>
-      <c r="G50" s="130"/>
-      <c r="H50" s="173"/>
-      <c r="I50" s="174"/>
-      <c r="J50" s="174"/>
-      <c r="K50" s="175"/>
+      <c r="D50" s="58"/>
+      <c r="E50" s="59"/>
+      <c r="F50" s="59"/>
+      <c r="G50" s="59"/>
+      <c r="H50" s="53"/>
+      <c r="I50" s="54"/>
+      <c r="J50" s="54"/>
+      <c r="K50" s="55"/>
     </row>
     <row r="51" spans="1:11" s="1" customFormat="1" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="135" t="s">
+      <c r="A51" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="B51" s="136"/>
-      <c r="C51" s="136"/>
-      <c r="D51" s="136"/>
-      <c r="E51" s="136"/>
-      <c r="F51" s="136"/>
-      <c r="G51" s="136"/>
-      <c r="H51" s="136"/>
-      <c r="I51" s="137"/>
-      <c r="J51" s="137"/>
-      <c r="K51" s="138"/>
+      <c r="B51" s="107"/>
+      <c r="C51" s="107"/>
+      <c r="D51" s="107"/>
+      <c r="E51" s="107"/>
+      <c r="F51" s="107"/>
+      <c r="G51" s="107"/>
+      <c r="H51" s="107"/>
+      <c r="I51" s="108"/>
+      <c r="J51" s="108"/>
+      <c r="K51" s="109"/>
     </row>
     <row r="52" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="117" t="s">
+      <c r="A52" s="116" t="s">
         <v>16</v>
       </c>
-      <c r="B52" s="118"/>
-      <c r="C52" s="119"/>
-      <c r="D52" s="119"/>
-      <c r="E52" s="119"/>
-      <c r="F52" s="119"/>
-      <c r="G52" s="119"/>
-      <c r="H52" s="119"/>
-      <c r="I52" s="119"/>
-      <c r="J52" s="119"/>
-      <c r="K52" s="120"/>
+      <c r="B52" s="117"/>
+      <c r="C52" s="118"/>
+      <c r="D52" s="118"/>
+      <c r="E52" s="118"/>
+      <c r="F52" s="118"/>
+      <c r="G52" s="118"/>
+      <c r="H52" s="118"/>
+      <c r="I52" s="118"/>
+      <c r="J52" s="118"/>
+      <c r="K52" s="119"/>
     </row>
     <row r="53" spans="1:11" s="1" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="15"/>
@@ -3003,20 +3322,20 @@
       <c r="K53" s="16"/>
     </row>
     <row r="54" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="114" t="s">
+      <c r="A54" s="113" t="s">
         <v>17</v>
       </c>
-      <c r="B54" s="115"/>
-      <c r="C54" s="115"/>
-      <c r="D54" s="115"/>
-      <c r="E54" s="115"/>
-      <c r="G54" s="115" t="s">
+      <c r="B54" s="114"/>
+      <c r="C54" s="114"/>
+      <c r="D54" s="114"/>
+      <c r="E54" s="114"/>
+      <c r="G54" s="114" t="s">
         <v>31</v>
       </c>
-      <c r="H54" s="115"/>
-      <c r="I54" s="115"/>
-      <c r="J54" s="115"/>
-      <c r="K54" s="116"/>
+      <c r="H54" s="114"/>
+      <c r="I54" s="114"/>
+      <c r="J54" s="114"/>
+      <c r="K54" s="115"/>
     </row>
     <row r="55" spans="1:11" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="17"/>
@@ -3033,6 +3352,82 @@
     </row>
   </sheetData>
   <mergeCells count="92">
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="C43:K43"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E12:K12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E13:K13"/>
+    <mergeCell ref="D2:K3"/>
+    <mergeCell ref="E11:K11"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="G54:K54"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:K52"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="C44:K44"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="C42:K42"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A35:K35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="C36:K36"/>
+    <mergeCell ref="C37:K37"/>
+    <mergeCell ref="C38:K38"/>
+    <mergeCell ref="C39:K39"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="E49:G49"/>
+    <mergeCell ref="H49:K49"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C45:K45"/>
     <mergeCell ref="A34:K34"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="C27:K27"/>
@@ -3049,82 +3444,6 @@
     <mergeCell ref="E48:G48"/>
     <mergeCell ref="H48:K48"/>
     <mergeCell ref="C49:D49"/>
-    <mergeCell ref="E49:G49"/>
-    <mergeCell ref="H49:K49"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C45:K45"/>
-    <mergeCell ref="C36:K36"/>
-    <mergeCell ref="C37:K37"/>
-    <mergeCell ref="C38:K38"/>
-    <mergeCell ref="C39:K39"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="C42:K42"/>
-    <mergeCell ref="A17:K17"/>
-    <mergeCell ref="A35:K35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A51:H51"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="G54:K54"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="C52:K52"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A29:K29"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A23:K23"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="E13:K13"/>
-    <mergeCell ref="D2:K3"/>
-    <mergeCell ref="E11:K11"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="C43:K43"/>
-    <mergeCell ref="C44:K44"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="E12:K12"/>
-    <mergeCell ref="A13:D13"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -3133,4 +3452,827 @@
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F683090B-E632-40E2-8CAE-44FCAD04AC64}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P55"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="10" width="9.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.140625" customWidth="1"/>
+    <col min="12" max="12" width="5.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="24"/>
+    </row>
+    <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="25"/>
+      <c r="D2" s="152" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="152"/>
+      <c r="F2" s="152"/>
+      <c r="G2" s="152"/>
+      <c r="H2" s="152"/>
+      <c r="I2" s="152"/>
+      <c r="J2" s="152"/>
+      <c r="K2" s="153"/>
+    </row>
+    <row r="3" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="25"/>
+      <c r="D3" s="152"/>
+      <c r="E3" s="152"/>
+      <c r="F3" s="152"/>
+      <c r="G3" s="152"/>
+      <c r="H3" s="152"/>
+      <c r="I3" s="152"/>
+      <c r="J3" s="152"/>
+      <c r="K3" s="153"/>
+    </row>
+    <row r="4" spans="1:11" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="17"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="32" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="25"/>
+      <c r="K5" s="30"/>
+    </row>
+    <row r="6" spans="1:11" s="6" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="212" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="213"/>
+      <c r="C6" s="213"/>
+      <c r="D6" s="213"/>
+      <c r="E6" s="213"/>
+      <c r="F6" s="213"/>
+      <c r="G6" s="213"/>
+      <c r="H6" s="213"/>
+      <c r="I6" s="213"/>
+      <c r="J6" s="213"/>
+      <c r="K6" s="214"/>
+    </row>
+    <row r="7" spans="1:11" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="81" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="215"/>
+      <c r="F7" s="216"/>
+      <c r="G7" s="216"/>
+      <c r="H7" s="216"/>
+      <c r="I7" s="216"/>
+      <c r="J7" s="216"/>
+      <c r="K7" s="217"/>
+    </row>
+    <row r="8" spans="1:11" s="6" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="81" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="82"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="218"/>
+      <c r="F8" s="219"/>
+      <c r="G8" s="219"/>
+      <c r="H8" s="219"/>
+      <c r="I8" s="219"/>
+      <c r="J8" s="219"/>
+      <c r="K8" s="220"/>
+    </row>
+    <row r="9" spans="1:11" s="6" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="211"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="54"/>
+      <c r="G9" s="54"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
+      <c r="J9" s="54"/>
+      <c r="K9" s="55"/>
+    </row>
+    <row r="10" spans="1:11" s="6" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="51" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="127"/>
+      <c r="C10" s="127"/>
+      <c r="D10" s="127"/>
+      <c r="E10" s="127"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="127"/>
+      <c r="H10" s="127"/>
+      <c r="I10" s="127"/>
+      <c r="J10" s="127"/>
+      <c r="K10" s="128"/>
+    </row>
+    <row r="11" spans="1:11" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="181" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="182"/>
+      <c r="C11" s="182"/>
+      <c r="D11" s="182"/>
+      <c r="E11" s="182" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="182"/>
+      <c r="G11" s="182" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="182"/>
+      <c r="I11" s="182" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="182"/>
+      <c r="K11" s="183"/>
+    </row>
+    <row r="12" spans="1:11" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="184"/>
+      <c r="B12" s="185"/>
+      <c r="C12" s="185"/>
+      <c r="D12" s="186"/>
+      <c r="E12" s="187"/>
+      <c r="F12" s="188"/>
+      <c r="G12" s="187"/>
+      <c r="H12" s="188"/>
+      <c r="I12" s="187"/>
+      <c r="J12" s="189"/>
+      <c r="K12" s="190"/>
+    </row>
+    <row r="13" spans="1:11" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="184"/>
+      <c r="B13" s="185"/>
+      <c r="C13" s="185"/>
+      <c r="D13" s="186"/>
+      <c r="E13" s="187"/>
+      <c r="F13" s="188"/>
+      <c r="G13" s="187"/>
+      <c r="H13" s="188"/>
+      <c r="I13" s="187"/>
+      <c r="J13" s="189"/>
+      <c r="K13" s="190"/>
+    </row>
+    <row r="14" spans="1:11" s="6" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="191"/>
+      <c r="B14" s="192"/>
+      <c r="C14" s="192"/>
+      <c r="D14" s="193"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="79"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="79"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="78"/>
+      <c r="K14" s="80"/>
+    </row>
+    <row r="15" spans="1:11" s="6" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="31"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="194"/>
+    </row>
+    <row r="16" spans="1:11" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="51" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="127"/>
+      <c r="C16" s="127"/>
+      <c r="D16" s="127"/>
+      <c r="E16" s="127"/>
+      <c r="F16" s="127"/>
+      <c r="G16" s="127"/>
+      <c r="H16" s="127"/>
+      <c r="I16" s="127"/>
+      <c r="J16" s="127"/>
+      <c r="K16" s="128"/>
+    </row>
+    <row r="17" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="181" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="182"/>
+      <c r="C17" s="182" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="182"/>
+      <c r="E17" s="182"/>
+      <c r="F17" s="182" t="s">
+        <v>68</v>
+      </c>
+      <c r="G17" s="182"/>
+      <c r="H17" s="182" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" s="182"/>
+      <c r="J17" s="182" t="s">
+        <v>70</v>
+      </c>
+      <c r="K17" s="183"/>
+    </row>
+    <row r="18" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="195"/>
+      <c r="B18" s="196"/>
+      <c r="C18" s="120"/>
+      <c r="D18" s="120"/>
+      <c r="E18" s="120"/>
+      <c r="F18" s="120"/>
+      <c r="G18" s="120"/>
+      <c r="H18" s="197"/>
+      <c r="I18" s="197"/>
+      <c r="J18" s="120"/>
+      <c r="K18" s="121"/>
+    </row>
+    <row r="19" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="221"/>
+      <c r="B19" s="222"/>
+      <c r="C19" s="223"/>
+      <c r="D19" s="223"/>
+      <c r="E19" s="223"/>
+      <c r="F19" s="223"/>
+      <c r="G19" s="223"/>
+      <c r="H19" s="224"/>
+      <c r="I19" s="224"/>
+      <c r="J19" s="223"/>
+      <c r="K19" s="225"/>
+    </row>
+    <row r="20" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="126"/>
+      <c r="B20" s="126"/>
+      <c r="C20" s="120"/>
+      <c r="D20" s="120"/>
+      <c r="E20" s="120"/>
+      <c r="F20" s="120"/>
+      <c r="G20" s="120"/>
+      <c r="H20" s="197"/>
+      <c r="I20" s="197"/>
+      <c r="J20" s="120"/>
+      <c r="K20" s="121"/>
+    </row>
+    <row r="21" spans="1:16" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="211"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="54"/>
+      <c r="J21" s="54"/>
+      <c r="K21" s="55"/>
+    </row>
+    <row r="22" spans="1:16" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="127"/>
+      <c r="C22" s="127"/>
+      <c r="D22" s="127"/>
+      <c r="E22" s="127"/>
+      <c r="F22" s="127"/>
+      <c r="G22" s="127"/>
+      <c r="H22" s="127"/>
+      <c r="I22" s="127"/>
+      <c r="J22" s="127"/>
+      <c r="K22" s="128"/>
+    </row>
+    <row r="23" spans="1:16" s="1" customFormat="1" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="198" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="199"/>
+      <c r="C23" s="199"/>
+      <c r="D23" s="199"/>
+      <c r="E23" s="199"/>
+      <c r="F23" s="199" t="s">
+        <v>73</v>
+      </c>
+      <c r="G23" s="199"/>
+      <c r="H23" s="200" t="s">
+        <v>74</v>
+      </c>
+      <c r="I23" s="201"/>
+      <c r="J23" s="200" t="s">
+        <v>75</v>
+      </c>
+      <c r="K23" s="202"/>
+    </row>
+    <row r="24" spans="1:16" s="1" customFormat="1" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="195"/>
+      <c r="B24" s="203"/>
+      <c r="C24" s="203"/>
+      <c r="D24" s="203"/>
+      <c r="E24" s="196"/>
+      <c r="F24" s="120"/>
+      <c r="G24" s="120"/>
+      <c r="H24" s="187"/>
+      <c r="I24" s="188"/>
+      <c r="J24" s="187"/>
+      <c r="K24" s="190"/>
+    </row>
+    <row r="25" spans="1:16" s="1" customFormat="1" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="195"/>
+      <c r="B25" s="203"/>
+      <c r="C25" s="203"/>
+      <c r="D25" s="203"/>
+      <c r="E25" s="196"/>
+      <c r="F25" s="120"/>
+      <c r="G25" s="120"/>
+      <c r="H25" s="187"/>
+      <c r="I25" s="188"/>
+      <c r="J25" s="187"/>
+      <c r="K25" s="190"/>
+    </row>
+    <row r="26" spans="1:16" s="1" customFormat="1" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="140"/>
+      <c r="B26" s="141"/>
+      <c r="C26" s="141"/>
+      <c r="D26" s="141"/>
+      <c r="E26" s="143"/>
+      <c r="F26" s="112"/>
+      <c r="G26" s="112"/>
+      <c r="H26" s="204"/>
+      <c r="I26" s="205"/>
+      <c r="J26" s="204"/>
+      <c r="K26" s="206"/>
+    </row>
+    <row r="27" spans="1:16" s="1" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="207"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="194"/>
+    </row>
+    <row r="28" spans="1:16" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="51" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="127"/>
+      <c r="C28" s="127"/>
+      <c r="D28" s="127"/>
+      <c r="E28" s="127"/>
+      <c r="F28" s="127"/>
+      <c r="G28" s="127"/>
+      <c r="H28" s="127"/>
+      <c r="I28" s="127"/>
+      <c r="J28" s="127"/>
+      <c r="K28" s="128"/>
+    </row>
+    <row r="29" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="181" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="182"/>
+      <c r="C29" s="182"/>
+      <c r="D29" s="182"/>
+      <c r="E29" s="182" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" s="182"/>
+      <c r="G29" s="182" t="s">
+        <v>79</v>
+      </c>
+      <c r="H29" s="182"/>
+      <c r="I29" s="182" t="s">
+        <v>80</v>
+      </c>
+      <c r="J29" s="182"/>
+      <c r="K29" s="183"/>
+    </row>
+    <row r="30" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="125"/>
+      <c r="B30" s="126"/>
+      <c r="C30" s="126"/>
+      <c r="D30" s="126"/>
+      <c r="E30" s="120"/>
+      <c r="F30" s="120"/>
+      <c r="G30" s="208"/>
+      <c r="H30" s="208"/>
+      <c r="I30" s="120"/>
+      <c r="J30" s="120"/>
+      <c r="K30" s="121"/>
+    </row>
+    <row r="31" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="125"/>
+      <c r="B31" s="126"/>
+      <c r="C31" s="126"/>
+      <c r="D31" s="126"/>
+      <c r="E31" s="129"/>
+      <c r="F31" s="129"/>
+      <c r="G31" s="209"/>
+      <c r="H31" s="209"/>
+      <c r="I31" s="120"/>
+      <c r="J31" s="120"/>
+      <c r="K31" s="121"/>
+      <c r="P31" s="2"/>
+    </row>
+    <row r="32" spans="1:16" s="1" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="123"/>
+      <c r="B32" s="124"/>
+      <c r="C32" s="124"/>
+      <c r="D32" s="124"/>
+      <c r="E32" s="124"/>
+      <c r="F32" s="124"/>
+      <c r="G32" s="210"/>
+      <c r="H32" s="210"/>
+      <c r="I32" s="112"/>
+      <c r="J32" s="112"/>
+      <c r="K32" s="122"/>
+    </row>
+    <row r="33" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33"/>
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
+      <c r="I33"/>
+      <c r="J33"/>
+      <c r="K33"/>
+    </row>
+    <row r="34" spans="1:11" s="1" customFormat="1" ht="3" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34"/>
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="J34"/>
+      <c r="K34"/>
+    </row>
+    <row r="35" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35"/>
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35"/>
+      <c r="F35"/>
+      <c r="G35"/>
+      <c r="H35"/>
+      <c r="I35"/>
+      <c r="J35"/>
+      <c r="K35"/>
+    </row>
+    <row r="36" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36"/>
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36"/>
+      <c r="F36"/>
+      <c r="G36"/>
+      <c r="H36"/>
+      <c r="I36"/>
+      <c r="J36"/>
+      <c r="K36"/>
+    </row>
+    <row r="37" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37"/>
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37"/>
+      <c r="F37"/>
+      <c r="G37"/>
+      <c r="H37"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37"/>
+    </row>
+    <row r="38" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38"/>
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+      <c r="E38"/>
+      <c r="F38"/>
+      <c r="G38"/>
+      <c r="H38"/>
+      <c r="I38"/>
+      <c r="J38"/>
+      <c r="K38"/>
+    </row>
+    <row r="39" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39"/>
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+      <c r="E39"/>
+      <c r="F39"/>
+      <c r="G39"/>
+      <c r="H39"/>
+      <c r="I39"/>
+      <c r="J39"/>
+      <c r="K39"/>
+    </row>
+    <row r="40" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40"/>
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40"/>
+      <c r="E40"/>
+      <c r="F40"/>
+      <c r="G40"/>
+      <c r="H40"/>
+      <c r="I40"/>
+      <c r="J40"/>
+      <c r="K40"/>
+    </row>
+    <row r="41" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41"/>
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41"/>
+      <c r="E41"/>
+      <c r="F41"/>
+      <c r="G41"/>
+      <c r="H41"/>
+      <c r="I41"/>
+      <c r="J41"/>
+      <c r="K41"/>
+    </row>
+    <row r="42" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42"/>
+      <c r="B42"/>
+      <c r="C42"/>
+      <c r="D42"/>
+      <c r="E42"/>
+      <c r="F42"/>
+      <c r="G42"/>
+      <c r="H42"/>
+      <c r="I42"/>
+      <c r="J42"/>
+      <c r="K42"/>
+    </row>
+    <row r="43" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43"/>
+      <c r="B43"/>
+      <c r="C43"/>
+      <c r="D43"/>
+      <c r="E43"/>
+      <c r="F43"/>
+      <c r="G43"/>
+      <c r="H43"/>
+      <c r="I43"/>
+      <c r="J43"/>
+      <c r="K43"/>
+    </row>
+    <row r="44" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44"/>
+      <c r="B44"/>
+      <c r="C44"/>
+      <c r="D44"/>
+      <c r="E44"/>
+      <c r="F44"/>
+      <c r="G44"/>
+      <c r="H44"/>
+      <c r="I44"/>
+      <c r="J44"/>
+      <c r="K44"/>
+    </row>
+    <row r="45" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45"/>
+      <c r="B45"/>
+      <c r="C45"/>
+      <c r="D45"/>
+      <c r="E45"/>
+      <c r="F45"/>
+      <c r="G45"/>
+      <c r="H45"/>
+      <c r="I45"/>
+      <c r="J45"/>
+      <c r="K45"/>
+    </row>
+    <row r="46" spans="1:11" s="1" customFormat="1" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46"/>
+      <c r="B46"/>
+      <c r="C46"/>
+      <c r="D46"/>
+      <c r="E46"/>
+      <c r="F46"/>
+      <c r="G46"/>
+      <c r="H46"/>
+      <c r="I46"/>
+      <c r="J46"/>
+      <c r="K46"/>
+    </row>
+    <row r="47" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47"/>
+      <c r="B47"/>
+      <c r="C47"/>
+      <c r="D47"/>
+      <c r="E47"/>
+      <c r="F47"/>
+      <c r="G47"/>
+      <c r="H47"/>
+      <c r="I47"/>
+      <c r="J47"/>
+      <c r="K47"/>
+    </row>
+    <row r="48" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48"/>
+      <c r="B48"/>
+      <c r="C48"/>
+      <c r="D48"/>
+      <c r="E48"/>
+      <c r="F48"/>
+      <c r="G48"/>
+      <c r="H48"/>
+      <c r="I48"/>
+      <c r="J48"/>
+      <c r="K48"/>
+    </row>
+    <row r="49" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49"/>
+      <c r="B49"/>
+      <c r="C49"/>
+      <c r="D49"/>
+      <c r="E49"/>
+      <c r="F49"/>
+      <c r="G49"/>
+      <c r="H49"/>
+      <c r="I49"/>
+      <c r="J49"/>
+      <c r="K49"/>
+    </row>
+    <row r="50" spans="1:11" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50"/>
+      <c r="B50"/>
+      <c r="C50"/>
+      <c r="D50"/>
+      <c r="E50"/>
+      <c r="F50"/>
+      <c r="G50"/>
+      <c r="H50"/>
+      <c r="I50"/>
+      <c r="J50"/>
+      <c r="K50"/>
+    </row>
+    <row r="51" spans="1:11" s="1" customFormat="1" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51"/>
+      <c r="B51"/>
+      <c r="C51"/>
+      <c r="D51"/>
+      <c r="E51"/>
+      <c r="F51"/>
+      <c r="G51"/>
+      <c r="H51"/>
+      <c r="I51"/>
+      <c r="J51"/>
+      <c r="K51"/>
+    </row>
+    <row r="52" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="53" spans="1:11" s="1" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53"/>
+      <c r="B53"/>
+      <c r="C53"/>
+      <c r="D53"/>
+      <c r="E53"/>
+      <c r="F53"/>
+      <c r="G53"/>
+      <c r="H53"/>
+      <c r="I53"/>
+      <c r="J53"/>
+      <c r="K53"/>
+    </row>
+    <row r="54" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="55" spans="1:11" ht="4.5" customHeight="1" x14ac:dyDescent="0.2"/>
+  </sheetData>
+  <mergeCells count="80">
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="E7:K7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E8:K8"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="D2:K3"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.31496062992125984" bottom="0.31496062992125984" header="0.19685039370078741" footer="0.19685039370078741"/>
+  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>